<commit_message>
feat(appconfig): ASSISTANT v1.0.18 sans bundles Graph dans Git
</commit_message>
<xml_diff>
--- a/templates/BilanDeCollecte.xlsx
+++ b/templates/BilanDeCollecte.xlsx
@@ -524,15 +524,15 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>0</xdr:col>
-      <xdr:colOff>104760</xdr:colOff>
+      <xdr:colOff>82800</xdr:colOff>
       <xdr:row>0</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
+      <xdr:rowOff>74160</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>2</xdr:col>
-      <xdr:colOff>532800</xdr:colOff>
+      <xdr:colOff>510480</xdr:colOff>
       <xdr:row>1</xdr:row>
-      <xdr:rowOff>176760</xdr:rowOff>
+      <xdr:rowOff>250560</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -546,8 +546,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="104760" y="0"/>
-          <a:ext cx="807120" cy="376920"/>
+          <a:off x="82800" y="74160"/>
+          <a:ext cx="806760" cy="376560"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -754,7 +754,7 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="1" width="3.42"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="10" style="1" width="5.14"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="14" style="1" width="4.57"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="15" min="15" style="1" width="7.73"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="15" min="15" style="1" width="8.02"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16" min="16" style="1" width="4.42"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="17" min="17" style="1" width="2"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="18" min="18" style="1" width="11.14"/>
@@ -786,7 +786,7 @@
       <c r="R1" s="6"/>
       <c r="S1" s="6"/>
     </row>
-    <row r="2" s="7" customFormat="true" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="2" s="7" customFormat="true" ht="26.6" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="2"/>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>

</xml_diff>